<commit_message>
refactor(ranking): separate academic score from real market PnL
</commit_message>
<xml_diff>
--- a/PlanilhaChaves.xlsx
+++ b/PlanilhaChaves.xlsx
@@ -3,9 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
-  <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25000" windowHeight="10000" firstSheet="0" activeTab="0"/>
-  </bookViews>
   <sheets>
     <sheet sheetId="1" name="Worksheet" state="visible" r:id="rId4"/>
   </sheets>
@@ -14,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>ID</t>
   </si>
@@ -25,16 +22,13 @@
     <t>CHAVE_PK</t>
   </si>
   <si>
-    <t>Valentim</t>
+    <t>33039</t>
+  </si>
+  <si>
+    <t>Otoniel Emanuel</t>
   </si>
   <si>
     <t>0x8b3a350cf5c34c9194ca85829a2df0ec3153be0318b5e2d3348e872092edffba</t>
-  </si>
-  <si>
-    <t>Otoniel</t>
-  </si>
-  <si>
-    <t>0x92db14e403b83dfe3df233f83dfa3a0d7096f21ca9b0d6d6b8d88b2b4ec1564e</t>
   </si>
 </sst>
 </file>
@@ -234,20 +228,16 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -369,18 +359,54 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -394,29 +420,16 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>33031</v>
+      <c r="A2" t="s">
+        <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>33038</v>
-      </c>
-      <c r="B3" t="s">
         <v>5</v>
-      </c>
-      <c r="C3" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="default" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: align ranking and bots with weighted PnL evaluation
</commit_message>
<xml_diff>
--- a/PlanilhaChaves.xlsx
+++ b/PlanilhaChaves.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>ID</t>
   </si>
@@ -29,6 +29,15 @@
   </si>
   <si>
     <t>0x8b3a350cf5c34c9194ca85829a2df0ec3153be0318b5e2d3348e872092edffba</t>
+  </si>
+  <si>
+    <t>11111</t>
+  </si>
+  <si>
+    <t>Teste</t>
+  </si>
+  <si>
+    <t>0x92db14e403b83dfe3df233f83dfa3a0d7096f21ca9b0d6d6b8d88b2b4ec1564e</t>
   </si>
 </sst>
 </file>
@@ -405,7 +414,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -430,6 +439,17 @@
         <v>5</v>
       </c>
     </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
local chart & update .gitignore
</commit_message>
<xml_diff>
--- a/PlanilhaChaves.xlsx
+++ b/PlanilhaChaves.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>ID</t>
   </si>
@@ -22,22 +22,40 @@
     <t>CHAVE_PK</t>
   </si>
   <si>
+    <t>33031</t>
+  </si>
+  <si>
+    <t>Valentim</t>
+  </si>
+  <si>
+    <t>0x8b3a350cf5c34c9194ca85829a2df0ec3153be0318b5e2d3348e872092edffba</t>
+  </si>
+  <si>
     <t>33039</t>
   </si>
   <si>
-    <t>Otoniel Emanuel</t>
-  </si>
-  <si>
-    <t>0x8b3a350cf5c34c9194ca85829a2df0ec3153be0318b5e2d3348e872092edffba</t>
-  </si>
-  <si>
-    <t>11111</t>
-  </si>
-  <si>
-    <t>Teste</t>
+    <t>Otoniel</t>
   </si>
   <si>
     <t>0x92db14e403b83dfe3df233f83dfa3a0d7096f21ca9b0d6d6b8d88b2b4ec1564e</t>
+  </si>
+  <si>
+    <t>22029</t>
+  </si>
+  <si>
+    <t>Azevedo</t>
+  </si>
+  <si>
+    <t>0x4bbbf85ce3377467afe5d46f804f221813b2bb87f24d81f60f1fcdbf7cbf4356</t>
+  </si>
+  <si>
+    <t>00000</t>
+  </si>
+  <si>
+    <t>NOVA</t>
+  </si>
+  <si>
+    <t>0xdbda1821b80551c9d65939329250298aa3472ba22feea921c0cf5d620ea67b97</t>
   </si>
 </sst>
 </file>
@@ -414,7 +432,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -450,6 +468,28 @@
         <v>8</v>
       </c>
     </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>